<commit_message>
Updated code to generate news summarization
</commit_message>
<xml_diff>
--- a/NewsLinks.xlsx
+++ b/NewsLinks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Workspace\PyCharmWorkspace\NewsSummarizer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C00366-1FBC-46E4-9865-BA28669B0CD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A737BE4F-4615-49EE-ADB2-3DC9E5F082FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{3FDC74BA-37A5-4E49-9CE0-B752517C2BB7}"/>
+    <workbookView xWindow="2415" yWindow="-13800" windowWidth="21600" windowHeight="11235" xr2:uid="{3FDC74BA-37A5-4E49-9CE0-B752517C2BB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -452,62 +452,62 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BB648F2-73F2-4729-BCED-C6578472C75E}">
   <dimension ref="A1:A11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="55.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="55.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>

</xml_diff>